<commit_message>
docs: execution_surfaces.yaml parses again (two new scalars quoted); EXECUTION_SURFACES.xlsx rebuilt from it (verify OK)
The previous commit appended R47–R53 with two plain scalars containing ": " (YAML reads that as a nested key), so the spec did not
load, the docs tests failed and the committed workbook was the previous build. Both scalars are quoted; the workbook is rebuilt
(Layers 4/4/10, steps 2/5/6 unchanged; 53 remediation rows, 8 equality checks).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QedX4KjNg2eSfF8fZ1UQ6b
</commit_message>
<xml_diff>
--- a/docs/EXECUTION_SURFACES.xlsx
+++ b/docs/EXECUTION_SURFACES.xlsx
@@ -878,7 +878,7 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>A · Cloud Run function (deploy.sh → gcloud run deploy --function, Scheduler OIDC, Secret Manager, BigQuery MERGE)</t>
+          <t>A · Cloud Run function (deploy.sh → gcloud run deploy --function, Scheduler OIDC, Secret Manager, BigQuery MERGE) — operator surfaces: Cloud Shell runbook docs/RUNBOOK_CLOUD_SHELL.md and the Vertex AI Workbench notebook notebooks/cloudbq_deploy_and_witness.ipynb (same deploy.sh)</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
@@ -1039,9 +1039,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>`deploy.sh secret`: Secret Manager hubspot-token (create or versions add from $HUBSPOT_TOKEN in the shell, never in .env), accessor
-for the SA; `deploy.sh deploy` pins --set-secrets HUBSPOT_TOKEN=hubspot-token:${SECRET_VERSION} (empty → newest enabled version
-number resolved at deploy time, never the literal "latest"); optional DELIVERY_WEBHOOK_TOKEN from $DELIVERY_WEBHOOK_TOKEN_SECRET.</t>
+          <t>`deploy.sh secret`: Secret Manager hubspot-token (create or versions add from $HUBSPOT_TOKEN typed into the shell — never in .env, check-env refuses it), accessor for the SA; prints the version NUMBER; `deploy.sh deploy` pins --set-secrets HUBSPOT_TOKEN=hubspot-token:${SECRET_VERSION} (empty → newest enabled version number resolved with value(name.basename()) at deploy time, never the literal "latest" and never the resource path, R47); optional DELIVERY_WEBHOOK_TOKEN from $DELIVERY_WEBHOOK_TOKEN_SECRET.</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1077,8 +1075,7 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>deploy.sh refuses nothing here but resolves the version number (read); deploy_job.sh refuses a missing version (DRYRUN=1 run);
-secrets.sh DRYRUN=1 lists the three secrets. Secrets created: not yet — first authenticated run.</t>
+          <t>deploy.sh secret_version() resolves the version NUMBER with value(name.basename()) — value(name) returned projects/…/versions/N and would have been rejected by --set-secrets (R47, fixed 574e954, DRYRUN=1 prints the corrected command); deploy_job.sh refuses a missing version (DRYRUN=1 run); secrets.sh DRYRUN=1 lists the three secrets. Secrets created: not yet — first authenticated run.</t>
         </is>
       </c>
     </row>
@@ -1095,9 +1092,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>`deploy.sh invoker`: two Cloud Scheduler HTTP jobs new-deals-SEALSQ "0 7 * * 1" and new-deals-ICALPS "20 7 * * 1" --time-zone
-Europe/Zurich, GET $URL?entity=…, --oidc-service-account-email new-deals-fn@, --oidc-token-audience $URL, --attempt-deadline 600s,
---max-retry-attempts 3, create-or-update, created PAUSED; `deploy.sh enable` resumes.</t>
+          <t>`deploy.sh invoker`: two Cloud Scheduler HTTP jobs new-deals-SEALSQ "0 7 * * 1" and new-deals-ICALPS "20 7 * * 1" --time-zone Europe/Zurich, GET $URL?entity=…, --oidc-service-account-email new-deals-fn@, --oidc-token-audience $URL, --attempt-deadline 600s, --max-retry-attempts 3, create-or-update, created PAUSED; `deploy.sh enable` resumes only PAUSED jobs and `pause` only ENABLED ones (idempotent, R49). Cloud Scheduler is offered in europe-west6 (locations page, 2026-10-16).</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1551,9 +1546,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>`deploy.sh dry`: ?dry_run=1 for both entities; main.py builds the BigQuery client in dry mode, reads watermark + warehouse twins,
-skips MERGE, history, watermark, run row and delivery; payload carries dry_run: true; the step asserts rows_written == 0 and prints
-rows/dup/hot/window. Nothing is written; the lease is not taken.</t>
+          <t>`deploy.sh dry`: ?dry_run=1 for both entities; main.py builds the BigQuery client in dry mode, reads watermark + warehouse twins, skips MERGE, history, watermark, run row and delivery; payload carries dry_run: true; the step asserts rows_written == 0 and prints rows/dup/hot/window. curl -sSf: an HTTP 403 (caller lacks run.invoker) or 409 (lease held) fails the gate instead of passing a JSON error as a payload (R50). Nothing is written; the lease is not taken. Same gate from the Workbench notebook (cells 3.8 and 4.6) and the Cloud Shell runbook Phase 7.</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1609,9 +1602,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>`deploy.sh replay ENTITY FROM_ISO`: UPDATE report_state SET watermark = TIMESTAMP 'FROM', updated_at = now WHERE report_id =
-'NEW_DEALS_&lt;entity&gt;' then `deploy.sh run ENTITY`; MERGE dedupes; day1_* frozen so historical scores survive; new_deals_history slice
-for the new run_ts; the first run with no watermark looks back FIRST_RUN_DAYS.</t>
+          <t>`deploy.sh replay ENTITY FROM_ISO`: UPDATE report_state SET watermark = TIMESTAMP 'FROM', updated_at = now WHERE report_id = 'NEW_DEALS_&lt;entity&gt;' then `deploy.sh run ENTITY`; MERGE dedupes; day1_* frozen so historical scores survive; new_deals_history slice for the new run_ts; the first run with no watermark looks back FIRST_RUN_DAYS. replay is the idempotency check of the runbook (FROM = window.query_start of the first run); a second `run` opens the next window instead (R52).</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1725,9 +1716,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Private service (--no-allow-unauthenticated); `deploy.sh invoker` binds roles/run.invoker to new-deals-fn@ for the Scheduler's OIDC
-token (humans need run.invoker for `deploy.sh dry`/`run`); SA roles: bigquery.jobUser (project), dataEditor (dataset DCL),
-secretmanager.secretAccessor (hubspot-token); HubSpot read-only private app.</t>
+          <t>Private service (--no-allow-unauthenticated); `deploy.sh invoker` binds roles/run.invoker to new-deals-fn@ for the Scheduler's OIDC token; humans need run.invoker for `deploy.sh dry`/`run` (Owner/Editor have it); when gcloud's active account is a service account (Workbench instance, VM) `invoke` mints the ID token with --audiences $URL, which Cloud Run requires for service accounts (R48); SA roles: bigquery.jobUser (project), dataEditor (dataset DCL — on the whole dataset, e.g. mrload), secretmanager.secretAccessor (hubspot-token); HubSpot read-only private app.</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1976,7 +1965,7 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>A · Cloud Run function (deploy.sh → gcloud run deploy --function, Scheduler OIDC, Secret Manager, BigQuery MERGE) — cell</t>
+          <t>A · Cloud Run function (deploy.sh → gcloud run deploy --function, Scheduler OIDC, Secret Manager, BigQuery MERGE) — operator surfaces: Cloud Shell runbook docs/RUNBOOK_CLOUD_SHELL.md and the Vertex AI Workbench notebook notebooks/cloudbq_deploy_and_witness.ipynb (same deploy.sh) — cell</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
@@ -2181,7 +2170,7 @@
       <c r="C6" s="4" t="inlineStr"/>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>HUBSPOT_TOKEN=… deploy.sh secret — hubspot-token create or versions add, secretAccessor for the SA; prints the version to pin in .env SECRET_VERSION</t>
+          <t>IFS= read -rsp … HUBSPOT_TOKEN; HUBSPOT_TOKEN="$HUBSPOT_TOKEN" deploy.sh secret — hubspot-token create or versions add (a version per run), secretAccessor for the SA; prints the version NUMBER (value(name.basename()), R47) to pin in .env SECRET_VERSION (optional: deploy resolves the newest enabled number)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -2308,7 +2297,7 @@
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>deploy.sh dry — curl $URL?entity=SEALSQ&amp;dry_run=1 and ICALPS with an identity token; asserts rows_written == 0 and dry_run true; prints rows/dup/hot/window</t>
+          <t>deploy.sh dry — curl -sSf $URL?entity=SEALSQ&amp;dry_run=1 and ICALPS with the caller's identity token (a service account's carries audience = $URL, R48); asserts rows_written == 0 and dry_run true; an HTTP 403 (caller lacks run.invoker) or 409 (lease held) fails the step (R50); prints rows/dup/hot/window</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -2353,7 +2342,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>deploy.sh run SEALSQ then deploy.sh run ICALPS — one live window run each; prints report_id, run_timestamp, window, row_count, rows_written, duplicate_suspects, day1_hot</t>
+          <t>deploy.sh run SEALSQ then deploy.sh run ICALPS — one live window run each (the first without a watermark looks back FIRST_RUN_DAYS); prints report_id, run_timestamp, window, row_count, rows_written, duplicate_suspects, day1_hot; refuses an error payload or one without rows_written (R50); each run moves the watermark — the idempotency check is step 13 replay, not a second run (R52)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -2398,7 +2387,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>deploy.sh enable — gcloud scheduler jobs resume new-deals-SEALSQ / -ICALPS</t>
+          <t>deploy.sh enable — gcloud scheduler jobs resume new-deals-SEALSQ / -ICALPS, only those in state PAUSED (idempotent, R49); pause likewise only ENABLED jobs</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -2525,7 +2514,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>deploy.sh replay SEALSQ 2026-09-01T00:00:00Z — UPDATE report_state SET watermark = TIMESTAMP '…' WHERE report_id = 'NEW_DEALS_SEALSQ' then deploy.sh run SEALSQ</t>
+          <t>deploy.sh replay SEALSQ FROM_ISO — UPDATE report_state SET watermark = TIMESTAMP 'FROM' WHERE report_id = 'NEW_DEALS_SEALSQ' then deploy.sh run SEALSQ; the runbook's idempotency check with FROM = window.query_start of the first run (R52): probe counts unchanged</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -2565,7 +2554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4316,6 +4305,265 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>R47</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Pre-run review (2026-10-16): deploy.sh secret_version() read the Secret Manager version with --format value(name), i.e. projects/N/secrets/hubspot-token/versions/V; `deploy` would have passed that path to --set-secrets and Cloud Run rejects it</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>gcloud's own table uses name.basename(); value(name) is the raw resource name.</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>deploy.sh lines 86 and 91 use --format 'value(name.basename())' (the version number); the `secret` hint prints the number.</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>fixed in 574e954 — DRYRUN=1 deploy.sh deploy prints value(name.basename()); live deploy not yet — first authenticated run</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>R48</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Pre-run review: from a Vertex AI Workbench instance or any VM whose gcloud account is a service account, `gcloud auth print-identity-token` carries gcloud's client id as audience; Cloud Run requires the service URL for service-account tokens, so `dry`/`run` would fail with 401/403 on that surface</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>deploy.sh invoke() minted the token without --audiences; only a person's token is accepted as is.</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>invoke() reads the active account; a *.gserviceaccount.com account gets --audiences "$u"; the notebook's cell 4.6 chooses by ADC type (user → gcloud token, service account → fetch_id_token(audience = URL)).</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>fixed in 574e954 / e88c27a (code read; DRYRUN=1 prints the account lookup); live call not yet — first authenticated run</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>R49</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Pre-run review: `deploy.sh enable` after a successful enable exited non-zero — the Scheduler API refuses to resume a job that is not PAUSED; same for pause; contradicted the header's "re-running a step is safe"</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>resume/pause were unconditional.</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>enable() resumes only jobs in state PAUSED, pause() only ENABLED ones (job_state helper); the header names the steps that are not no-ops (secret adds a version, run moves the watermark).</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>fixed in 574e954 (DRYRUN=1 enable/pause rehearsed); live not yet — first authenticated run</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>R50</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Pre-run review: `run` could not tell success from the function's 409 "lease held" or any JSON error body — curl without -f printed {"report_id": …} and exited 0 while nothing was written; `dry` would die with a JSONDecodeError on a 403 instead of the status</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>L11</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>invoke() used curl -sS; live() printed whatever keys were present.</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>curl -sSf (HTTP 4xx/5xx fail the step with the status); live() asserts no "error" key and a rows_written key; the runbook lists the status → cause table (403 caller lacks run.invoker, 500 + HubSpot 401 in logs, 500 + Not found table, 409 lease).</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>fixed in 574e954 (bash -n, DRYRUN=1 dry/run); live not yet — first authenticated run</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>R51</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Pre-run review: tests/test_hot_score.py emit_sql() wrote bare NULLs; a struct column that is NULL in every row of the UNNEST is typed INT64, so SAFE_CAST(… AS TIMESTAMP) and the STRING UDF parameters fail — impossible on the 15 golden vectors, likely on live deals (notes_last_updated, revenue_state often all NULL)</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>A C</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>BigQuery supertype rule for NULL-only literals; sql_literal() also left backslashes unescaped.</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>sql_literal(v, typ) emits CAST(NULL AS STRING|FLOAT64|BOOL) and escapes backslashes; tests/hot_score_vectors.sql regenerated; the notebook's live-parity cell reuses emit_sql unchanged.</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>fixed in 574e954 (python3 tests/test_hot_score.py: constants OK · python vectors OK · JS port OK); the SQL itself not yet executed — first authenticated run</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>R52</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Operator runbook draft: "BQ_LOCATION stays EU, fine for europe-west6" (the BigQuery location is independent of the Cloud Run region — it must equal the existing dataset's location), a second `run SEALSQ` as the idempotency check (each run moves the watermark, so it opens the next window), a 403 on `dry` attributed to the `invoker` step (dry uses the operator's identity), portal 49610528 vs 9201667</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>L11</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>The runbook was drafted from the sequence without the state model; the portal id came from an earlier draft.</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>docs/RUNBOOK_CLOUD_SHELL.md — Phase 2 checks `bq show` location == BQ_LOCATION (mrload was created in EU by mir-load run_pass1.sh); Phase 7 uses `replay SEALSQ "$FROM"` with FROM = window.query_start of the first run; 403 → the caller''s run.invoker; portal 9201667 confirmed as the hub id of the connected HubSpot account.</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>this commit (docs); PASS1_SEQUENCE.md corrected the same way in e88c27a</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>R53</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Operator runbook draft: Phase 3 ran python3 tests/*.py in Cloud Shell, whose Python has no functions-framework / google-cloud-bigquery / flask, so the offline rehearsal would have failed on import</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>main.py imports functions_framework at import time; the tests import main.</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>a virtualenv in $HOME (persists in Cloud Shell): python3 -m venv ~/.venvs/cloudbq &amp;&amp; pip install -r cloud_function_new_deals/requirements.txt pyyaml pytest; the Workbench notebook installs the same into its kernel.</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>this commit (docs); the CI job installs the same requirements before pytest (green)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4327,7 +4575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4350,7 +4598,7 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>A · Cloud Run function (deploy.sh → gcloud run deploy --function, Scheduler OIDC, Secret Manager, BigQuery MERGE) — cell</t>
+          <t>A · Cloud Run function (deploy.sh → gcloud run deploy --function, Scheduler OIDC, Secret Manager, BigQuery MERGE) — operator surfaces: Cloud Shell runbook docs/RUNBOOK_CLOUD_SHELL.md and the Vertex AI Workbench notebook notebooks/cloudbq_deploy_and_witness.ipynb (same deploy.sh) — cell</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
@@ -4550,6 +4798,33 @@
       <c r="E8" s="4" t="inlineStr">
         <is>
           <t>XLSX rows == row_count == rows of new_deals_last_7d for the same window; a zero-row week sends the text-only "no new deals" mail (B1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>probe from two operator surfaces (lane A)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>the two `probe` queries run by deploy.sh (bq CLI, Cloud Shell runbook Phase 7) and by the Workbench notebook cell 4.5 (BigQuery Python client) against the same tables</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>deploy.sh probe — SELECT entity, COUNT(*) n, COUNTIF(day1_hot_flag) hot, COUNTIF(duplicate_suspect) dup, MIN(createdate), MAX(createdate) FROM new_deals GROUP BY entity; last 10 new_deals_runs</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>n/a — same lane, two surfaces: notebooks/cloudbq_deploy_and_witness.ipynb cell 4.5 runs the identical SQL through bigquery.Client and prints job id, bytes processed, slot ms</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>identical rows and counts from both surfaces (job ids differ); the notebook additionally shows hot_score_v1 reproducing the 15 golden vectors and main.hot_score agreeing with it</t>
         </is>
       </c>
     </row>

</xml_diff>